<commit_message>
EFO 3.88, DO Feb 26
</commit_message>
<xml_diff>
--- a/data-raw/metadata_phen_oncox.xlsx
+++ b/data-raw/metadata_phen_oncox.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__phenOncoX/phenOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4653FA7F-509E-BD42-A2BA-36E6BE26EF94}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF31A19E-30F0-0E4A-A4AD-1B6DBEBD045F}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="2180" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
@@ -153,10 +153,10 @@
     <t>2025_10_03</t>
   </si>
   <si>
-    <t>v2026-02-02</t>
-  </si>
-  <si>
-    <t>v3.87.0</t>
+    <t>v2026-02-28</t>
+  </si>
+  <si>
+    <t>v3.88.0</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
May 2026 releas - qmd vignette
</commit_message>
<xml_diff>
--- a/data-raw/metadata_phen_oncox.xlsx
+++ b/data-raw/metadata_phen_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__phenOncoX/phenOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF31A19E-30F0-0E4A-A4AD-1B6DBEBD045F}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E44BF6D-7F88-8142-BB13-CEB5C96561E8}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="2180" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="6700" yWindow="3120" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="phen_oncox" sheetId="5" r:id="rId1"/>
@@ -153,10 +153,10 @@
     <t>2025_10_03</t>
   </si>
   <si>
-    <t>v2026-02-28</t>
-  </si>
-  <si>
-    <t>v3.88.0</t>
+    <t>v3.90.0</t>
+  </si>
+  <si>
+    <t>v2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -639,7 +639,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
@@ -665,7 +665,7 @@
         <v>14</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
update DO and fix wrong one-to-many primary site mappings
</commit_message>
<xml_diff>
--- a/data-raw/metadata_phen_oncox.xlsx
+++ b/data-raw/metadata_phen_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__phenOncoX/phenOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E44BF6D-7F88-8142-BB13-CEB5C96561E8}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7FD7A72-F791-9E46-BF2E-9E5ECB2E59B4}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6700" yWindow="3120" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="920" yWindow="3120" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="phen_oncox" sheetId="5" r:id="rId1"/>
@@ -156,7 +156,7 @@
     <t>v3.90.0</t>
   </si>
   <si>
-    <t>v2026-04-30</t>
+    <t>v2026-05-30</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
updated EFO and DO
</commit_message>
<xml_diff>
--- a/data-raw/metadata_phen_oncox.xlsx
+++ b/data-raw/metadata_phen_oncox.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__phenOncoX/phenOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7FD7A72-F791-9E46-BF2E-9E5ECB2E59B4}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FCDA147-F530-5A43-9369-74DD97E88D7D}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="920" yWindow="3120" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
@@ -153,10 +153,10 @@
     <t>2025_10_03</t>
   </si>
   <si>
-    <t>v3.90.0</t>
-  </si>
-  <si>
-    <t>v2026-05-30</t>
+    <t>v3.91.0</t>
+  </si>
+  <si>
+    <t>v2026-06-30</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
DO august 2026, EFO 3.93
</commit_message>
<xml_diff>
--- a/data-raw/metadata_phen_oncox.xlsx
+++ b/data-raw/metadata_phen_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__phenOncoX/phenOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FCDA147-F530-5A43-9369-74DD97E88D7D}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C664126E-2637-C945-8686-3BEDE9E08A8D}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="920" yWindow="3120" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="2300" yWindow="7960" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="phen_oncox" sheetId="5" r:id="rId1"/>
@@ -153,10 +153,10 @@
     <t>2025_10_03</t>
   </si>
   <si>
-    <t>v3.91.0</t>
-  </si>
-  <si>
-    <t>v2026-06-30</t>
+    <t>v3.93.0</t>
+  </si>
+  <si>
+    <t>v2026-08-31</t>
   </si>
 </sst>
 </file>

</xml_diff>